<commit_message>
Enhance Playwright configuration for Chromium. Added launch options for maximized window and non-headless mode.
</commit_message>
<xml_diff>
--- a/MyNotes/Playwright cheatsheet.xlsx
+++ b/MyNotes/Playwright cheatsheet.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="I:\YT Classes and Practice\Playwright SDET QA Pavan 2025\MyNotes\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8355A78D-EC64-45C0-8EBB-3A950B4E1166}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7F0797E7-4A1B-4AAD-A9E8-FFF72E08E09D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="2" xr2:uid="{EE043035-96D4-4599-856B-8BD9C43ACC17}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{EE043035-96D4-4599-856B-8BD9C43ACC17}"/>
   </bookViews>
   <sheets>
     <sheet name="Playwright built-in methods" sheetId="2" r:id="rId1"/>
@@ -22,7 +22,6 @@
     <sheet name="Playwright Commands" sheetId="5" r:id="rId7"/>
   </sheets>
   <calcPr calcId="191029"/>
-  <fileRecoveryPr repairLoad="1"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
@@ -1026,9 +1025,6 @@
     <t>Opens the generated HTML report.</t>
   </si>
   <si>
-    <t>Creates a new isolated browser context.</t>
-  </si>
-  <si>
     <t>Closes the browser instance.</t>
   </si>
   <si>
@@ -2242,6 +2238,9 @@
   </si>
   <si>
     <t>Scrolls element into view</t>
+  </si>
+  <si>
+    <t>Creates a new isolated browser session.</t>
   </si>
 </sst>
 </file>
@@ -2416,14 +2415,11 @@
     <xf numFmtId="0" fontId="1" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="3" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="3" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="3" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
+    <xf numFmtId="0" fontId="1" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="4" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
@@ -2452,11 +2448,14 @@
     <xf numFmtId="0" fontId="1" fillId="3" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -2828,7 +2827,7 @@
         <v>32</v>
       </c>
       <c r="E3" s="2" t="s">
-        <v>327</v>
+        <v>732</v>
       </c>
     </row>
     <row r="4" spans="2:5" x14ac:dyDescent="0.3">
@@ -2840,7 +2839,7 @@
         <v>34</v>
       </c>
       <c r="E4" s="2" t="s">
-        <v>328</v>
+        <v>327</v>
       </c>
     </row>
     <row r="5" spans="2:5" x14ac:dyDescent="0.3">
@@ -2852,7 +2851,7 @@
         <v>36</v>
       </c>
       <c r="E5" s="2" t="s">
-        <v>329</v>
+        <v>328</v>
       </c>
     </row>
     <row r="6" spans="2:5" x14ac:dyDescent="0.3">
@@ -2864,7 +2863,7 @@
         <v>38</v>
       </c>
       <c r="E6" s="2" t="s">
-        <v>330</v>
+        <v>329</v>
       </c>
     </row>
     <row r="7" spans="2:5" x14ac:dyDescent="0.3">
@@ -2876,7 +2875,7 @@
         <v>40</v>
       </c>
       <c r="E7" s="2" t="s">
-        <v>331</v>
+        <v>330</v>
       </c>
     </row>
     <row r="8" spans="2:5" x14ac:dyDescent="0.3">
@@ -2890,7 +2889,7 @@
         <v>43</v>
       </c>
       <c r="E8" s="2" t="s">
-        <v>332</v>
+        <v>331</v>
       </c>
     </row>
     <row r="9" spans="2:5" x14ac:dyDescent="0.3">
@@ -2902,7 +2901,7 @@
         <v>45</v>
       </c>
       <c r="E9" s="2" t="s">
-        <v>333</v>
+        <v>332</v>
       </c>
     </row>
     <row r="10" spans="2:5" x14ac:dyDescent="0.3">
@@ -2914,7 +2913,7 @@
         <v>47</v>
       </c>
       <c r="E10" s="2" t="s">
-        <v>334</v>
+        <v>333</v>
       </c>
     </row>
     <row r="11" spans="2:5" x14ac:dyDescent="0.3">
@@ -2926,7 +2925,7 @@
         <v>49</v>
       </c>
       <c r="E11" s="2" t="s">
-        <v>335</v>
+        <v>334</v>
       </c>
     </row>
     <row r="12" spans="2:5" x14ac:dyDescent="0.3">
@@ -2938,7 +2937,7 @@
         <v>51</v>
       </c>
       <c r="E12" s="2" t="s">
-        <v>336</v>
+        <v>335</v>
       </c>
     </row>
     <row r="13" spans="2:5" x14ac:dyDescent="0.3">
@@ -2950,7 +2949,7 @@
         <v>53</v>
       </c>
       <c r="E13" s="2" t="s">
-        <v>337</v>
+        <v>336</v>
       </c>
     </row>
     <row r="14" spans="2:5" x14ac:dyDescent="0.3">
@@ -2962,7 +2961,7 @@
         <v>55</v>
       </c>
       <c r="E14" s="2" t="s">
-        <v>338</v>
+        <v>337</v>
       </c>
     </row>
     <row r="15" spans="2:5" x14ac:dyDescent="0.3">
@@ -2976,7 +2975,7 @@
         <v>58</v>
       </c>
       <c r="E15" s="2" t="s">
-        <v>339</v>
+        <v>338</v>
       </c>
     </row>
     <row r="16" spans="2:5" x14ac:dyDescent="0.3">
@@ -2988,7 +2987,7 @@
         <v>60</v>
       </c>
       <c r="E16" s="2" t="s">
-        <v>340</v>
+        <v>339</v>
       </c>
     </row>
     <row r="17" spans="2:5" x14ac:dyDescent="0.3">
@@ -3000,7 +2999,7 @@
         <v>62</v>
       </c>
       <c r="E17" s="2" t="s">
-        <v>341</v>
+        <v>340</v>
       </c>
     </row>
     <row r="18" spans="2:5" x14ac:dyDescent="0.3">
@@ -3012,7 +3011,7 @@
         <v>64</v>
       </c>
       <c r="E18" s="2" t="s">
-        <v>342</v>
+        <v>341</v>
       </c>
     </row>
     <row r="19" spans="2:5" x14ac:dyDescent="0.3">
@@ -3024,7 +3023,7 @@
         <v>66</v>
       </c>
       <c r="E19" s="2" t="s">
-        <v>343</v>
+        <v>342</v>
       </c>
     </row>
     <row r="20" spans="2:5" x14ac:dyDescent="0.3">
@@ -3036,7 +3035,7 @@
         <v>68</v>
       </c>
       <c r="E20" s="2" t="s">
-        <v>344</v>
+        <v>343</v>
       </c>
     </row>
     <row r="21" spans="2:5" x14ac:dyDescent="0.3">
@@ -3048,7 +3047,7 @@
         <v>70</v>
       </c>
       <c r="E21" s="2" t="s">
-        <v>345</v>
+        <v>344</v>
       </c>
     </row>
     <row r="22" spans="2:5" x14ac:dyDescent="0.3">
@@ -3060,7 +3059,7 @@
         <v>72</v>
       </c>
       <c r="E22" s="2" t="s">
-        <v>346</v>
+        <v>345</v>
       </c>
     </row>
     <row r="23" spans="2:5" x14ac:dyDescent="0.3">
@@ -3072,7 +3071,7 @@
         <v>74</v>
       </c>
       <c r="E23" s="2" t="s">
-        <v>347</v>
+        <v>346</v>
       </c>
     </row>
     <row r="24" spans="2:5" x14ac:dyDescent="0.3">
@@ -3084,7 +3083,7 @@
         <v>76</v>
       </c>
       <c r="E24" s="2" t="s">
-        <v>348</v>
+        <v>347</v>
       </c>
     </row>
     <row r="25" spans="2:5" x14ac:dyDescent="0.3">
@@ -3096,7 +3095,7 @@
         <v>78</v>
       </c>
       <c r="E25" s="2" t="s">
-        <v>349</v>
+        <v>348</v>
       </c>
     </row>
     <row r="26" spans="2:5" x14ac:dyDescent="0.3">
@@ -3108,7 +3107,7 @@
         <v>80</v>
       </c>
       <c r="E26" s="2" t="s">
-        <v>350</v>
+        <v>349</v>
       </c>
     </row>
     <row r="27" spans="2:5" x14ac:dyDescent="0.3">
@@ -3120,7 +3119,7 @@
         <v>82</v>
       </c>
       <c r="E27" s="2" t="s">
-        <v>351</v>
+        <v>350</v>
       </c>
     </row>
     <row r="28" spans="2:5" x14ac:dyDescent="0.3">
@@ -3132,7 +3131,7 @@
         <v>83</v>
       </c>
       <c r="E28" s="2" t="s">
-        <v>352</v>
+        <v>351</v>
       </c>
     </row>
     <row r="29" spans="2:5" x14ac:dyDescent="0.3">
@@ -3146,7 +3145,7 @@
         <v>85</v>
       </c>
       <c r="E29" s="2" t="s">
-        <v>353</v>
+        <v>352</v>
       </c>
     </row>
     <row r="30" spans="2:5" x14ac:dyDescent="0.3">
@@ -3158,7 +3157,7 @@
         <v>86</v>
       </c>
       <c r="E30" s="2" t="s">
-        <v>354</v>
+        <v>353</v>
       </c>
     </row>
     <row r="31" spans="2:5" x14ac:dyDescent="0.3">
@@ -3170,7 +3169,7 @@
         <v>87</v>
       </c>
       <c r="E31" s="2" t="s">
-        <v>355</v>
+        <v>354</v>
       </c>
     </row>
     <row r="32" spans="2:5" x14ac:dyDescent="0.3">
@@ -3182,7 +3181,7 @@
         <v>88</v>
       </c>
       <c r="E32" s="2" t="s">
-        <v>356</v>
+        <v>355</v>
       </c>
     </row>
     <row r="33" spans="2:5" x14ac:dyDescent="0.3">
@@ -3194,7 +3193,7 @@
         <v>90</v>
       </c>
       <c r="E33" s="2" t="s">
-        <v>357</v>
+        <v>356</v>
       </c>
     </row>
     <row r="34" spans="2:5" x14ac:dyDescent="0.3">
@@ -3206,7 +3205,7 @@
         <v>92</v>
       </c>
       <c r="E34" s="2" t="s">
-        <v>358</v>
+        <v>357</v>
       </c>
     </row>
     <row r="35" spans="2:5" x14ac:dyDescent="0.3">
@@ -3218,7 +3217,7 @@
         <v>94</v>
       </c>
       <c r="E35" s="2" t="s">
-        <v>359</v>
+        <v>358</v>
       </c>
     </row>
     <row r="36" spans="2:5" x14ac:dyDescent="0.3">
@@ -3230,7 +3229,7 @@
         <v>96</v>
       </c>
       <c r="E36" s="2" t="s">
-        <v>360</v>
+        <v>359</v>
       </c>
     </row>
     <row r="37" spans="2:5" x14ac:dyDescent="0.3">
@@ -3242,7 +3241,7 @@
         <v>98</v>
       </c>
       <c r="E37" s="2" t="s">
-        <v>361</v>
+        <v>360</v>
       </c>
     </row>
     <row r="38" spans="2:5" x14ac:dyDescent="0.3">
@@ -3254,7 +3253,7 @@
         <v>100</v>
       </c>
       <c r="E38" s="2" t="s">
-        <v>362</v>
+        <v>361</v>
       </c>
     </row>
     <row r="39" spans="2:5" x14ac:dyDescent="0.3">
@@ -3266,7 +3265,7 @@
         <v>102</v>
       </c>
       <c r="E39" s="2" t="s">
-        <v>363</v>
+        <v>362</v>
       </c>
     </row>
     <row r="40" spans="2:5" x14ac:dyDescent="0.3">
@@ -3278,7 +3277,7 @@
         <v>104</v>
       </c>
       <c r="E40" s="2" t="s">
-        <v>364</v>
+        <v>363</v>
       </c>
     </row>
     <row r="41" spans="2:5" x14ac:dyDescent="0.3">
@@ -3290,7 +3289,7 @@
         <v>106</v>
       </c>
       <c r="E41" s="2" t="s">
-        <v>365</v>
+        <v>364</v>
       </c>
     </row>
     <row r="42" spans="2:5" x14ac:dyDescent="0.3">
@@ -3302,7 +3301,7 @@
         <v>108</v>
       </c>
       <c r="E42" s="2" t="s">
-        <v>366</v>
+        <v>365</v>
       </c>
     </row>
     <row r="43" spans="2:5" x14ac:dyDescent="0.3">
@@ -3316,7 +3315,7 @@
         <v>110</v>
       </c>
       <c r="E43" s="2" t="s">
-        <v>367</v>
+        <v>366</v>
       </c>
     </row>
     <row r="44" spans="2:5" x14ac:dyDescent="0.3">
@@ -3328,7 +3327,7 @@
         <v>111</v>
       </c>
       <c r="E44" s="2" t="s">
-        <v>368</v>
+        <v>367</v>
       </c>
     </row>
     <row r="45" spans="2:5" x14ac:dyDescent="0.3">
@@ -3340,7 +3339,7 @@
         <v>112</v>
       </c>
       <c r="E45" s="2" t="s">
-        <v>369</v>
+        <v>368</v>
       </c>
     </row>
     <row r="46" spans="2:5" x14ac:dyDescent="0.3">
@@ -3352,7 +3351,7 @@
         <v>113</v>
       </c>
       <c r="E46" s="2" t="s">
-        <v>370</v>
+        <v>369</v>
       </c>
     </row>
     <row r="47" spans="2:5" x14ac:dyDescent="0.3">
@@ -3366,7 +3365,7 @@
         <v>115</v>
       </c>
       <c r="E47" s="2" t="s">
-        <v>371</v>
+        <v>370</v>
       </c>
     </row>
     <row r="48" spans="2:5" x14ac:dyDescent="0.3">
@@ -3378,7 +3377,7 @@
         <v>117</v>
       </c>
       <c r="E48" s="2" t="s">
-        <v>372</v>
+        <v>371</v>
       </c>
     </row>
     <row r="49" spans="2:5" x14ac:dyDescent="0.3">
@@ -3390,7 +3389,7 @@
         <v>119</v>
       </c>
       <c r="E49" s="2" t="s">
-        <v>373</v>
+        <v>372</v>
       </c>
     </row>
     <row r="50" spans="2:5" x14ac:dyDescent="0.3">
@@ -3402,7 +3401,7 @@
         <v>121</v>
       </c>
       <c r="E50" s="2" t="s">
-        <v>374</v>
+        <v>373</v>
       </c>
     </row>
     <row r="51" spans="2:5" x14ac:dyDescent="0.3">
@@ -3414,7 +3413,7 @@
         <v>123</v>
       </c>
       <c r="E51" s="2" t="s">
-        <v>375</v>
+        <v>374</v>
       </c>
     </row>
     <row r="52" spans="2:5" x14ac:dyDescent="0.3">
@@ -3426,7 +3425,7 @@
         <v>125</v>
       </c>
       <c r="E52" s="2" t="s">
-        <v>376</v>
+        <v>375</v>
       </c>
     </row>
   </sheetData>
@@ -3460,10 +3459,10 @@
   <sheetData>
     <row r="2" spans="2:8" x14ac:dyDescent="0.3">
       <c r="B2" s="1" t="s">
-        <v>413</v>
+        <v>412</v>
       </c>
       <c r="C2" s="1" t="s">
-        <v>481</v>
+        <v>480</v>
       </c>
       <c r="D2" s="1" t="s">
         <v>0</v>
@@ -3475,18 +3474,18 @@
         <v>234</v>
       </c>
       <c r="G2" s="8" t="s">
+        <v>536</v>
+      </c>
+      <c r="H2" s="8" t="s">
         <v>537</v>
       </c>
-      <c r="H2" s="8" t="s">
-        <v>538</v>
-      </c>
     </row>
     <row r="3" spans="2:8" ht="31.2" x14ac:dyDescent="0.3">
-      <c r="B3" s="28" t="s">
-        <v>482</v>
-      </c>
-      <c r="C3" s="19" t="s">
-        <v>414</v>
+      <c r="B3" s="27" t="s">
+        <v>481</v>
+      </c>
+      <c r="C3" s="30" t="s">
+        <v>413</v>
       </c>
       <c r="D3" s="10" t="s">
         <v>12</v>
@@ -3495,75 +3494,75 @@
         <v>13</v>
       </c>
       <c r="F3" s="10" t="s">
-        <v>483</v>
+        <v>482</v>
       </c>
       <c r="G3" s="11" t="s">
-        <v>596</v>
+        <v>595</v>
       </c>
       <c r="H3" s="11" t="s">
-        <v>539</v>
+        <v>538</v>
       </c>
     </row>
     <row r="4" spans="2:8" x14ac:dyDescent="0.3">
-      <c r="B4" s="29"/>
-      <c r="C4" s="20"/>
+      <c r="B4" s="28"/>
+      <c r="C4" s="31"/>
       <c r="D4" s="10" t="s">
         <v>14</v>
       </c>
       <c r="E4" s="10" t="s">
+        <v>414</v>
+      </c>
+      <c r="F4" s="10" t="s">
+        <v>483</v>
+      </c>
+      <c r="G4" s="11" t="s">
+        <v>596</v>
+      </c>
+      <c r="H4" s="11" t="s">
+        <v>539</v>
+      </c>
+    </row>
+    <row r="5" spans="2:8" ht="31.2" x14ac:dyDescent="0.3">
+      <c r="B5" s="28"/>
+      <c r="C5" s="31"/>
+      <c r="D5" s="10" t="s">
         <v>415</v>
-      </c>
-      <c r="F4" s="10" t="s">
-        <v>484</v>
-      </c>
-      <c r="G4" s="11" t="s">
-        <v>597</v>
-      </c>
-      <c r="H4" s="11" t="s">
-        <v>540</v>
-      </c>
-    </row>
-    <row r="5" spans="2:8" ht="31.2" x14ac:dyDescent="0.3">
-      <c r="B5" s="29"/>
-      <c r="C5" s="20"/>
-      <c r="D5" s="10" t="s">
-        <v>416</v>
       </c>
       <c r="E5" s="10" t="s">
         <v>15</v>
       </c>
       <c r="F5" s="10" t="s">
-        <v>485</v>
+        <v>484</v>
       </c>
       <c r="G5" s="11" t="s">
-        <v>598</v>
+        <v>597</v>
       </c>
       <c r="H5" s="11" t="s">
-        <v>541</v>
+        <v>540</v>
       </c>
     </row>
     <row r="6" spans="2:8" ht="31.2" x14ac:dyDescent="0.3">
-      <c r="B6" s="29"/>
-      <c r="C6" s="20"/>
+      <c r="B6" s="28"/>
+      <c r="C6" s="31"/>
       <c r="D6" s="10" t="s">
         <v>16</v>
       </c>
       <c r="E6" s="10" t="s">
-        <v>417</v>
+        <v>416</v>
       </c>
       <c r="F6" s="10" t="s">
-        <v>486</v>
+        <v>485</v>
       </c>
       <c r="G6" s="11" t="s">
-        <v>599</v>
+        <v>598</v>
       </c>
       <c r="H6" s="11" t="s">
-        <v>542</v>
+        <v>541</v>
       </c>
     </row>
     <row r="7" spans="2:8" ht="31.2" x14ac:dyDescent="0.3">
-      <c r="B7" s="29"/>
-      <c r="C7" s="20"/>
+      <c r="B7" s="28"/>
+      <c r="C7" s="31"/>
       <c r="D7" s="10" t="s">
         <v>17</v>
       </c>
@@ -3571,37 +3570,37 @@
         <v>18</v>
       </c>
       <c r="F7" s="10" t="s">
+        <v>486</v>
+      </c>
+      <c r="G7" s="11" t="s">
+        <v>599</v>
+      </c>
+      <c r="H7" s="11" t="s">
+        <v>542</v>
+      </c>
+    </row>
+    <row r="8" spans="2:8" x14ac:dyDescent="0.3">
+      <c r="B8" s="28"/>
+      <c r="C8" s="31"/>
+      <c r="D8" s="10" t="s">
+        <v>417</v>
+      </c>
+      <c r="E8" s="10" t="s">
+        <v>418</v>
+      </c>
+      <c r="F8" s="10" t="s">
         <v>487</v>
       </c>
-      <c r="G7" s="11" t="s">
-        <v>600</v>
-      </c>
-      <c r="H7" s="11" t="s">
+      <c r="G8" s="11" t="s">
         <v>543</v>
       </c>
-    </row>
-    <row r="8" spans="2:8" x14ac:dyDescent="0.3">
-      <c r="B8" s="29"/>
-      <c r="C8" s="20"/>
-      <c r="D8" s="10" t="s">
-        <v>418</v>
-      </c>
-      <c r="E8" s="10" t="s">
-        <v>419</v>
-      </c>
-      <c r="F8" s="10" t="s">
-        <v>488</v>
-      </c>
-      <c r="G8" s="11" t="s">
-        <v>544</v>
-      </c>
       <c r="H8" s="11" t="s">
-        <v>539</v>
+        <v>538</v>
       </c>
     </row>
     <row r="9" spans="2:8" x14ac:dyDescent="0.3">
-      <c r="B9" s="29"/>
-      <c r="C9" s="21"/>
+      <c r="B9" s="28"/>
+      <c r="C9" s="32"/>
       <c r="D9" s="10" t="s">
         <v>7</v>
       </c>
@@ -3609,39 +3608,39 @@
         <v>19</v>
       </c>
       <c r="F9" s="10" t="s">
-        <v>489</v>
+        <v>488</v>
       </c>
       <c r="G9" s="11" t="s">
-        <v>545</v>
+        <v>544</v>
       </c>
       <c r="H9" s="11" t="s">
-        <v>539</v>
+        <v>538</v>
       </c>
     </row>
     <row r="10" spans="2:8" x14ac:dyDescent="0.3">
-      <c r="B10" s="29"/>
-      <c r="C10" s="19" t="s">
-        <v>420</v>
+      <c r="B10" s="28"/>
+      <c r="C10" s="30" t="s">
+        <v>419</v>
       </c>
       <c r="D10" s="10" t="s">
-        <v>536</v>
+        <v>535</v>
       </c>
       <c r="E10" s="10" t="s">
         <v>9</v>
       </c>
       <c r="F10" s="10" t="s">
-        <v>534</v>
+        <v>533</v>
       </c>
       <c r="G10" s="11" t="s">
-        <v>546</v>
+        <v>545</v>
       </c>
       <c r="H10" s="11" t="s">
-        <v>539</v>
+        <v>538</v>
       </c>
     </row>
     <row r="11" spans="2:8" x14ac:dyDescent="0.3">
-      <c r="B11" s="29"/>
-      <c r="C11" s="20"/>
+      <c r="B11" s="28"/>
+      <c r="C11" s="31"/>
       <c r="D11" s="10" t="s">
         <v>8</v>
       </c>
@@ -3649,58 +3648,58 @@
         <v>10</v>
       </c>
       <c r="F11" s="10" t="s">
-        <v>535</v>
+        <v>534</v>
       </c>
       <c r="G11" s="11" t="s">
+        <v>546</v>
+      </c>
+      <c r="H11" s="11" t="s">
         <v>547</v>
       </c>
-      <c r="H11" s="11" t="s">
+    </row>
+    <row r="12" spans="2:8" x14ac:dyDescent="0.3">
+      <c r="B12" s="28"/>
+      <c r="C12" s="32"/>
+      <c r="D12" s="10" t="s">
+        <v>420</v>
+      </c>
+      <c r="E12" s="10" t="s">
+        <v>421</v>
+      </c>
+      <c r="F12" s="10" t="s">
+        <v>489</v>
+      </c>
+      <c r="G12" s="11" t="s">
         <v>548</v>
       </c>
-    </row>
-    <row r="12" spans="2:8" x14ac:dyDescent="0.3">
-      <c r="B12" s="29"/>
-      <c r="C12" s="21"/>
-      <c r="D12" s="10" t="s">
-        <v>421</v>
-      </c>
-      <c r="E12" s="10" t="s">
+      <c r="H12" s="11" t="s">
+        <v>547</v>
+      </c>
+    </row>
+    <row r="13" spans="2:8" ht="46.8" x14ac:dyDescent="0.3">
+      <c r="B13" s="28"/>
+      <c r="C13" s="30" t="s">
         <v>422</v>
       </c>
-      <c r="F12" s="10" t="s">
-        <v>490</v>
-      </c>
-      <c r="G12" s="11" t="s">
-        <v>549</v>
-      </c>
-      <c r="H12" s="11" t="s">
-        <v>548</v>
-      </c>
-    </row>
-    <row r="13" spans="2:8" ht="46.8" x14ac:dyDescent="0.3">
-      <c r="B13" s="29"/>
-      <c r="C13" s="19" t="s">
+      <c r="D13" s="10" t="s">
         <v>423</v>
-      </c>
-      <c r="D13" s="10" t="s">
-        <v>424</v>
       </c>
       <c r="E13" s="10" t="s">
         <v>21</v>
       </c>
       <c r="F13" s="10" t="s">
-        <v>491</v>
+        <v>490</v>
       </c>
       <c r="G13" s="11" t="s">
-        <v>601</v>
+        <v>600</v>
       </c>
       <c r="H13" s="11" t="s">
-        <v>550</v>
+        <v>549</v>
       </c>
     </row>
     <row r="14" spans="2:8" x14ac:dyDescent="0.3">
-      <c r="B14" s="29"/>
-      <c r="C14" s="20"/>
+      <c r="B14" s="28"/>
+      <c r="C14" s="31"/>
       <c r="D14" s="10" t="s">
         <v>8</v>
       </c>
@@ -3708,78 +3707,78 @@
         <v>22</v>
       </c>
       <c r="F14" s="10" t="s">
-        <v>492</v>
+        <v>491</v>
       </c>
       <c r="G14" s="11" t="s">
-        <v>551</v>
+        <v>550</v>
       </c>
       <c r="H14" s="11" t="s">
-        <v>543</v>
+        <v>542</v>
       </c>
     </row>
     <row r="15" spans="2:8" x14ac:dyDescent="0.3">
-      <c r="B15" s="29"/>
-      <c r="C15" s="21"/>
+      <c r="B15" s="28"/>
+      <c r="C15" s="32"/>
       <c r="D15" s="10" t="s">
-        <v>421</v>
+        <v>420</v>
       </c>
       <c r="E15" s="10" t="s">
         <v>23</v>
       </c>
       <c r="F15" s="10" t="s">
-        <v>493</v>
+        <v>492</v>
       </c>
       <c r="G15" s="11" t="s">
-        <v>552</v>
+        <v>551</v>
       </c>
       <c r="H15" s="11" t="s">
-        <v>543</v>
+        <v>542</v>
       </c>
     </row>
     <row r="16" spans="2:8" x14ac:dyDescent="0.3">
-      <c r="B16" s="29"/>
-      <c r="C16" s="19" t="s">
-        <v>425</v>
+      <c r="B16" s="28"/>
+      <c r="C16" s="30" t="s">
+        <v>424</v>
       </c>
       <c r="D16" s="10" t="s">
         <v>20</v>
       </c>
       <c r="E16" s="10" t="s">
-        <v>426</v>
+        <v>425</v>
       </c>
       <c r="F16" s="10" t="s">
-        <v>494</v>
+        <v>493</v>
       </c>
       <c r="G16" s="11" t="s">
-        <v>602</v>
+        <v>601</v>
       </c>
       <c r="H16" s="11" t="s">
-        <v>553</v>
+        <v>552</v>
       </c>
     </row>
     <row r="17" spans="2:8" x14ac:dyDescent="0.3">
-      <c r="B17" s="29"/>
-      <c r="C17" s="21"/>
+      <c r="B17" s="28"/>
+      <c r="C17" s="32"/>
       <c r="D17" s="10" t="s">
         <v>8</v>
       </c>
       <c r="E17" s="10" t="s">
+        <v>426</v>
+      </c>
+      <c r="F17" s="10" t="s">
+        <v>494</v>
+      </c>
+      <c r="G17" s="11" t="s">
+        <v>553</v>
+      </c>
+      <c r="H17" s="11" t="s">
+        <v>552</v>
+      </c>
+    </row>
+    <row r="18" spans="2:8" x14ac:dyDescent="0.3">
+      <c r="B18" s="28"/>
+      <c r="C18" s="30" t="s">
         <v>427</v>
-      </c>
-      <c r="F17" s="10" t="s">
-        <v>495</v>
-      </c>
-      <c r="G17" s="11" t="s">
-        <v>554</v>
-      </c>
-      <c r="H17" s="11" t="s">
-        <v>553</v>
-      </c>
-    </row>
-    <row r="18" spans="2:8" x14ac:dyDescent="0.3">
-      <c r="B18" s="29"/>
-      <c r="C18" s="19" t="s">
-        <v>428</v>
       </c>
       <c r="D18" s="10" t="s">
         <v>20</v>
@@ -3788,18 +3787,18 @@
         <v>24</v>
       </c>
       <c r="F18" s="10" t="s">
-        <v>496</v>
+        <v>495</v>
       </c>
       <c r="G18" s="12" t="s">
-        <v>603</v>
+        <v>602</v>
       </c>
       <c r="H18" s="12" t="s">
-        <v>555</v>
+        <v>554</v>
       </c>
     </row>
     <row r="19" spans="2:8" x14ac:dyDescent="0.3">
-      <c r="B19" s="29"/>
-      <c r="C19" s="21"/>
+      <c r="B19" s="28"/>
+      <c r="C19" s="32"/>
       <c r="D19" s="10" t="s">
         <v>8</v>
       </c>
@@ -3807,121 +3806,121 @@
         <v>25</v>
       </c>
       <c r="F19" s="10" t="s">
-        <v>497</v>
+        <v>496</v>
       </c>
       <c r="G19" s="13" t="s">
+        <v>555</v>
+      </c>
+      <c r="H19" s="13" t="s">
         <v>556</v>
       </c>
-      <c r="H19" s="13" t="s">
-        <v>557</v>
-      </c>
     </row>
     <row r="20" spans="2:8" ht="31.2" x14ac:dyDescent="0.3">
-      <c r="B20" s="29"/>
+      <c r="B20" s="28"/>
       <c r="C20" s="10" t="s">
+        <v>428</v>
+      </c>
+      <c r="D20" s="10" t="s">
         <v>429</v>
-      </c>
-      <c r="D20" s="10" t="s">
-        <v>430</v>
       </c>
       <c r="E20" s="10" t="s">
         <v>26</v>
       </c>
       <c r="F20" s="10" t="s">
+        <v>497</v>
+      </c>
+      <c r="G20" s="11" t="s">
+        <v>603</v>
+      </c>
+      <c r="H20" s="11" t="s">
+        <v>557</v>
+      </c>
+    </row>
+    <row r="21" spans="2:8" x14ac:dyDescent="0.3">
+      <c r="B21" s="29"/>
+      <c r="C21" s="9" t="s">
+        <v>529</v>
+      </c>
+      <c r="D21" s="10" t="s">
+        <v>530</v>
+      </c>
+      <c r="E21" s="10" t="s">
+        <v>531</v>
+      </c>
+      <c r="F21" s="10" t="s">
+        <v>532</v>
+      </c>
+      <c r="G21" s="11" t="s">
+        <v>604</v>
+      </c>
+      <c r="H21" s="11" t="s">
+        <v>558</v>
+      </c>
+    </row>
+    <row r="22" spans="2:8" x14ac:dyDescent="0.3">
+      <c r="B22" s="24" t="s">
+        <v>430</v>
+      </c>
+      <c r="C22" s="21" t="s">
         <v>498</v>
-      </c>
-      <c r="G20" s="11" t="s">
-        <v>604</v>
-      </c>
-      <c r="H20" s="11" t="s">
-        <v>558</v>
-      </c>
-    </row>
-    <row r="21" spans="2:8" x14ac:dyDescent="0.3">
-      <c r="B21" s="30"/>
-      <c r="C21" s="9" t="s">
-        <v>530</v>
-      </c>
-      <c r="D21" s="10" t="s">
-        <v>531</v>
-      </c>
-      <c r="E21" s="10" t="s">
-        <v>532</v>
-      </c>
-      <c r="F21" s="10" t="s">
-        <v>533</v>
-      </c>
-      <c r="G21" s="11" t="s">
-        <v>605</v>
-      </c>
-      <c r="H21" s="11" t="s">
-        <v>559</v>
-      </c>
-    </row>
-    <row r="22" spans="2:8" x14ac:dyDescent="0.3">
-      <c r="B22" s="25" t="s">
-        <v>431</v>
-      </c>
-      <c r="C22" s="22" t="s">
-        <v>499</v>
       </c>
       <c r="D22" s="14" t="s">
         <v>1</v>
       </c>
       <c r="E22" s="14" t="s">
+        <v>431</v>
+      </c>
+      <c r="F22" s="14" t="s">
         <v>432</v>
       </c>
-      <c r="F22" s="14" t="s">
-        <v>433</v>
-      </c>
       <c r="G22" s="15" t="s">
+        <v>559</v>
+      </c>
+      <c r="H22" s="15" t="s">
         <v>560</v>
       </c>
-      <c r="H22" s="15" t="s">
-        <v>561</v>
-      </c>
     </row>
     <row r="23" spans="2:8" ht="31.2" x14ac:dyDescent="0.3">
-      <c r="B23" s="26"/>
-      <c r="C23" s="23"/>
+      <c r="B23" s="25"/>
+      <c r="C23" s="22"/>
       <c r="D23" s="14" t="s">
         <v>2</v>
       </c>
       <c r="E23" s="14" t="s">
+        <v>433</v>
+      </c>
+      <c r="F23" s="14" t="s">
+        <v>499</v>
+      </c>
+      <c r="G23" s="15" t="s">
+        <v>561</v>
+      </c>
+      <c r="H23" s="15" t="s">
+        <v>562</v>
+      </c>
+    </row>
+    <row r="24" spans="2:8" x14ac:dyDescent="0.3">
+      <c r="B24" s="25"/>
+      <c r="C24" s="23"/>
+      <c r="D24" s="14" t="s">
         <v>434</v>
       </c>
-      <c r="F23" s="14" t="s">
+      <c r="E24" s="14" t="s">
+        <v>435</v>
+      </c>
+      <c r="F24" s="14" t="s">
         <v>500</v>
       </c>
-      <c r="G23" s="15" t="s">
-        <v>562</v>
-      </c>
-      <c r="H23" s="15" t="s">
+      <c r="G24" s="15" t="s">
         <v>563</v>
       </c>
-    </row>
-    <row r="24" spans="2:8" x14ac:dyDescent="0.3">
-      <c r="B24" s="26"/>
-      <c r="C24" s="24"/>
-      <c r="D24" s="14" t="s">
-        <v>435</v>
-      </c>
-      <c r="E24" s="14" t="s">
-        <v>436</v>
-      </c>
-      <c r="F24" s="14" t="s">
-        <v>501</v>
-      </c>
-      <c r="G24" s="15" t="s">
+      <c r="H24" s="15" t="s">
         <v>564</v>
       </c>
-      <c r="H24" s="15" t="s">
-        <v>565</v>
-      </c>
     </row>
     <row r="25" spans="2:8" x14ac:dyDescent="0.3">
-      <c r="B25" s="26"/>
-      <c r="C25" s="22" t="s">
+      <c r="B25" s="25"/>
+      <c r="C25" s="21" t="s">
         <v>3</v>
       </c>
       <c r="D25" s="14" t="s">
@@ -3931,299 +3930,299 @@
         <v>4</v>
       </c>
       <c r="F25" s="14" t="s">
+        <v>501</v>
+      </c>
+      <c r="G25" s="15" t="s">
+        <v>565</v>
+      </c>
+      <c r="H25" s="15" t="s">
+        <v>566</v>
+      </c>
+    </row>
+    <row r="26" spans="2:8" x14ac:dyDescent="0.3">
+      <c r="B26" s="25"/>
+      <c r="C26" s="22"/>
+      <c r="D26" s="14" t="s">
         <v>502</v>
       </c>
-      <c r="G25" s="15" t="s">
-        <v>566</v>
-      </c>
-      <c r="H25" s="15" t="s">
+      <c r="E26" s="14" t="s">
+        <v>436</v>
+      </c>
+      <c r="F26" s="14" t="s">
+        <v>503</v>
+      </c>
+      <c r="G26" s="15" t="s">
+        <v>605</v>
+      </c>
+      <c r="H26" s="15" t="s">
         <v>567</v>
       </c>
     </row>
-    <row r="26" spans="2:8" x14ac:dyDescent="0.3">
-      <c r="B26" s="26"/>
-      <c r="C26" s="23"/>
-      <c r="D26" s="14" t="s">
-        <v>503</v>
-      </c>
-      <c r="E26" s="14" t="s">
-        <v>437</v>
-      </c>
-      <c r="F26" s="14" t="s">
+    <row r="27" spans="2:8" x14ac:dyDescent="0.3">
+      <c r="B27" s="25"/>
+      <c r="C27" s="22"/>
+      <c r="D27" s="14" t="s">
+        <v>471</v>
+      </c>
+      <c r="E27" s="14" t="s">
+        <v>438</v>
+      </c>
+      <c r="F27" s="14" t="s">
+        <v>473</v>
+      </c>
+      <c r="G27" s="15" t="s">
+        <v>606</v>
+      </c>
+      <c r="H27" s="15" t="s">
+        <v>568</v>
+      </c>
+    </row>
+    <row r="28" spans="2:8" x14ac:dyDescent="0.3">
+      <c r="B28" s="25"/>
+      <c r="C28" s="23"/>
+      <c r="D28" s="14" t="s">
         <v>504</v>
       </c>
-      <c r="G26" s="15" t="s">
-        <v>606</v>
-      </c>
-      <c r="H26" s="15" t="s">
+      <c r="E28" s="14" t="s">
+        <v>439</v>
+      </c>
+      <c r="F28" s="14" t="s">
+        <v>440</v>
+      </c>
+      <c r="G28" s="15" t="s">
+        <v>607</v>
+      </c>
+      <c r="H28" s="15" t="s">
         <v>568</v>
       </c>
     </row>
-    <row r="27" spans="2:8" x14ac:dyDescent="0.3">
-      <c r="B27" s="26"/>
-      <c r="C27" s="23"/>
-      <c r="D27" s="14" t="s">
-        <v>472</v>
-      </c>
-      <c r="E27" s="14" t="s">
-        <v>439</v>
-      </c>
-      <c r="F27" s="14" t="s">
-        <v>474</v>
-      </c>
-      <c r="G27" s="15" t="s">
-        <v>607</v>
-      </c>
-      <c r="H27" s="15" t="s">
+    <row r="29" spans="2:8" ht="31.2" x14ac:dyDescent="0.3">
+      <c r="B29" s="25"/>
+      <c r="C29" s="14" t="s">
+        <v>505</v>
+      </c>
+      <c r="D29" s="14" t="s">
+        <v>441</v>
+      </c>
+      <c r="E29" s="14" t="s">
+        <v>442</v>
+      </c>
+      <c r="F29" s="14" t="s">
+        <v>506</v>
+      </c>
+      <c r="G29" s="15" t="s">
         <v>569</v>
       </c>
-    </row>
-    <row r="28" spans="2:8" x14ac:dyDescent="0.3">
-      <c r="B28" s="26"/>
-      <c r="C28" s="24"/>
-      <c r="D28" s="14" t="s">
-        <v>505</v>
-      </c>
-      <c r="E28" s="14" t="s">
-        <v>440</v>
-      </c>
-      <c r="F28" s="14" t="s">
-        <v>441</v>
-      </c>
-      <c r="G28" s="15" t="s">
+      <c r="H29" s="15" t="s">
+        <v>570</v>
+      </c>
+    </row>
+    <row r="30" spans="2:8" x14ac:dyDescent="0.3">
+      <c r="B30" s="25"/>
+      <c r="C30" s="14" t="s">
+        <v>507</v>
+      </c>
+      <c r="D30" s="14" t="s">
+        <v>443</v>
+      </c>
+      <c r="E30" s="14" t="s">
+        <v>444</v>
+      </c>
+      <c r="F30" s="14" t="s">
+        <v>508</v>
+      </c>
+      <c r="G30" s="15" t="s">
+        <v>571</v>
+      </c>
+      <c r="H30" s="15" t="s">
+        <v>572</v>
+      </c>
+    </row>
+    <row r="31" spans="2:8" x14ac:dyDescent="0.3">
+      <c r="B31" s="25"/>
+      <c r="C31" s="14" t="s">
+        <v>507</v>
+      </c>
+      <c r="D31" s="14" t="s">
+        <v>445</v>
+      </c>
+      <c r="E31" s="14" t="s">
+        <v>446</v>
+      </c>
+      <c r="F31" s="14" t="s">
+        <v>509</v>
+      </c>
+      <c r="G31" s="15" t="s">
         <v>608</v>
       </c>
-      <c r="H28" s="15" t="s">
-        <v>569</v>
-      </c>
-    </row>
-    <row r="29" spans="2:8" ht="31.2" x14ac:dyDescent="0.3">
-      <c r="B29" s="26"/>
-      <c r="C29" s="14" t="s">
-        <v>506</v>
-      </c>
-      <c r="D29" s="14" t="s">
-        <v>442</v>
-      </c>
-      <c r="E29" s="14" t="s">
-        <v>443</v>
-      </c>
-      <c r="F29" s="14" t="s">
-        <v>507</v>
-      </c>
-      <c r="G29" s="15" t="s">
-        <v>570</v>
-      </c>
-      <c r="H29" s="15" t="s">
-        <v>571</v>
-      </c>
-    </row>
-    <row r="30" spans="2:8" x14ac:dyDescent="0.3">
-      <c r="B30" s="26"/>
-      <c r="C30" s="14" t="s">
-        <v>508</v>
-      </c>
-      <c r="D30" s="14" t="s">
-        <v>444</v>
-      </c>
-      <c r="E30" s="14" t="s">
-        <v>445</v>
-      </c>
-      <c r="F30" s="14" t="s">
-        <v>509</v>
-      </c>
-      <c r="G30" s="15" t="s">
-        <v>572</v>
-      </c>
-      <c r="H30" s="15" t="s">
+      <c r="H31" s="15" t="s">
         <v>573</v>
       </c>
     </row>
-    <row r="31" spans="2:8" x14ac:dyDescent="0.3">
-      <c r="B31" s="26"/>
-      <c r="C31" s="14" t="s">
-        <v>508</v>
-      </c>
-      <c r="D31" s="14" t="s">
-        <v>446</v>
-      </c>
-      <c r="E31" s="14" t="s">
+    <row r="32" spans="2:8" x14ac:dyDescent="0.3">
+      <c r="B32" s="25"/>
+      <c r="C32" s="21" t="s">
+        <v>5</v>
+      </c>
+      <c r="D32" s="14" t="s">
+        <v>510</v>
+      </c>
+      <c r="E32" s="14" t="s">
         <v>447</v>
       </c>
-      <c r="F31" s="14" t="s">
-        <v>510</v>
-      </c>
-      <c r="G31" s="15" t="s">
-        <v>609</v>
-      </c>
-      <c r="H31" s="15" t="s">
+      <c r="F32" s="14" t="s">
+        <v>448</v>
+      </c>
+      <c r="G32" s="15" t="s">
         <v>574</v>
       </c>
-    </row>
-    <row r="32" spans="2:8" x14ac:dyDescent="0.3">
-      <c r="B32" s="26"/>
-      <c r="C32" s="22" t="s">
-        <v>5</v>
-      </c>
-      <c r="D32" s="14" t="s">
+      <c r="H32" s="15" t="s">
+        <v>540</v>
+      </c>
+    </row>
+    <row r="33" spans="2:8" x14ac:dyDescent="0.3">
+      <c r="B33" s="25"/>
+      <c r="C33" s="22"/>
+      <c r="D33" s="14" t="s">
+        <v>449</v>
+      </c>
+      <c r="E33" s="14" t="s">
+        <v>450</v>
+      </c>
+      <c r="F33" s="14" t="s">
         <v>511</v>
       </c>
-      <c r="E32" s="14" t="s">
-        <v>448</v>
-      </c>
-      <c r="F32" s="14" t="s">
-        <v>449</v>
-      </c>
-      <c r="G32" s="15" t="s">
+      <c r="G33" s="15" t="s">
         <v>575</v>
       </c>
-      <c r="H32" s="15" t="s">
-        <v>541</v>
-      </c>
-    </row>
-    <row r="33" spans="2:8" x14ac:dyDescent="0.3">
-      <c r="B33" s="26"/>
-      <c r="C33" s="23"/>
-      <c r="D33" s="14" t="s">
-        <v>450</v>
-      </c>
-      <c r="E33" s="14" t="s">
+      <c r="H33" s="15" t="s">
+        <v>576</v>
+      </c>
+    </row>
+    <row r="34" spans="2:8" ht="31.2" x14ac:dyDescent="0.3">
+      <c r="B34" s="25"/>
+      <c r="C34" s="22"/>
+      <c r="D34" s="14" t="s">
         <v>451</v>
-      </c>
-      <c r="F33" s="14" t="s">
-        <v>512</v>
-      </c>
-      <c r="G33" s="15" t="s">
-        <v>576</v>
-      </c>
-      <c r="H33" s="15" t="s">
-        <v>577</v>
-      </c>
-    </row>
-    <row r="34" spans="2:8" ht="31.2" x14ac:dyDescent="0.3">
-      <c r="B34" s="26"/>
-      <c r="C34" s="23"/>
-      <c r="D34" s="14" t="s">
-        <v>452</v>
       </c>
       <c r="E34" s="14" t="s">
         <v>6</v>
       </c>
       <c r="F34" s="14" t="s">
+        <v>452</v>
+      </c>
+      <c r="G34" s="15" t="s">
+        <v>577</v>
+      </c>
+      <c r="H34" s="15" t="s">
+        <v>578</v>
+      </c>
+    </row>
+    <row r="35" spans="2:8" ht="31.2" x14ac:dyDescent="0.3">
+      <c r="B35" s="25"/>
+      <c r="C35" s="23"/>
+      <c r="D35" s="14" t="s">
         <v>453</v>
       </c>
-      <c r="G34" s="15" t="s">
+      <c r="E35" s="14" t="s">
+        <v>454</v>
+      </c>
+      <c r="F35" s="14" t="s">
+        <v>455</v>
+      </c>
+      <c r="G35" s="15" t="s">
+        <v>579</v>
+      </c>
+      <c r="H35" s="15" t="s">
         <v>578</v>
       </c>
-      <c r="H34" s="15" t="s">
-        <v>579</v>
-      </c>
-    </row>
-    <row r="35" spans="2:8" ht="31.2" x14ac:dyDescent="0.3">
-      <c r="B35" s="26"/>
-      <c r="C35" s="24"/>
-      <c r="D35" s="14" t="s">
-        <v>454</v>
-      </c>
-      <c r="E35" s="14" t="s">
-        <v>455</v>
-      </c>
-      <c r="F35" s="14" t="s">
+    </row>
+    <row r="36" spans="2:8" ht="31.2" x14ac:dyDescent="0.3">
+      <c r="B36" s="25"/>
+      <c r="C36" s="14" t="s">
+        <v>512</v>
+      </c>
+      <c r="D36" s="14" t="s">
+        <v>429</v>
+      </c>
+      <c r="E36" s="14" t="s">
         <v>456</v>
       </c>
-      <c r="G35" s="15" t="s">
+      <c r="F36" s="14" t="s">
+        <v>513</v>
+      </c>
+      <c r="G36" s="15" t="s">
+        <v>429</v>
+      </c>
+      <c r="H36" s="15" t="s">
         <v>580</v>
       </c>
-      <c r="H35" s="15" t="s">
-        <v>579</v>
-      </c>
-    </row>
-    <row r="36" spans="2:8" ht="31.2" x14ac:dyDescent="0.3">
-      <c r="B36" s="26"/>
-      <c r="C36" s="14" t="s">
-        <v>513</v>
-      </c>
-      <c r="D36" s="14" t="s">
-        <v>430</v>
-      </c>
-      <c r="E36" s="14" t="s">
+    </row>
+    <row r="37" spans="2:8" x14ac:dyDescent="0.3">
+      <c r="B37" s="26"/>
+      <c r="C37" s="14" t="s">
+        <v>514</v>
+      </c>
+      <c r="D37" s="14" t="s">
         <v>457</v>
       </c>
-      <c r="F36" s="14" t="s">
-        <v>514</v>
-      </c>
-      <c r="G36" s="15" t="s">
-        <v>430</v>
-      </c>
-      <c r="H36" s="15" t="s">
+      <c r="E37" s="14" t="s">
+        <v>458</v>
+      </c>
+      <c r="F37" s="14" t="s">
+        <v>515</v>
+      </c>
+      <c r="G37" s="15" t="s">
+        <v>609</v>
+      </c>
+      <c r="H37" s="15" t="s">
         <v>581</v>
       </c>
     </row>
-    <row r="37" spans="2:8" x14ac:dyDescent="0.3">
-      <c r="B37" s="27"/>
-      <c r="C37" s="14" t="s">
-        <v>515</v>
-      </c>
-      <c r="D37" s="14" t="s">
-        <v>458</v>
-      </c>
-      <c r="E37" s="14" t="s">
+    <row r="38" spans="2:8" x14ac:dyDescent="0.3">
+      <c r="B38" s="20" t="s">
         <v>459</v>
       </c>
-      <c r="F37" s="14" t="s">
+      <c r="C38" s="19" t="s">
         <v>516</v>
       </c>
-      <c r="G37" s="15" t="s">
-        <v>610</v>
-      </c>
-      <c r="H37" s="15" t="s">
-        <v>582</v>
-      </c>
-    </row>
-    <row r="38" spans="2:8" x14ac:dyDescent="0.3">
-      <c r="B38" s="32" t="s">
+      <c r="D38" s="10" t="s">
+        <v>517</v>
+      </c>
+      <c r="E38" s="10" t="s">
+        <v>461</v>
+      </c>
+      <c r="F38" s="10" t="s">
+        <v>462</v>
+      </c>
+      <c r="G38" s="11" t="s">
         <v>460</v>
       </c>
-      <c r="C38" s="31" t="s">
-        <v>517</v>
-      </c>
-      <c r="D38" s="10" t="s">
+      <c r="H38" s="11" t="s">
+        <v>538</v>
+      </c>
+    </row>
+    <row r="39" spans="2:8" x14ac:dyDescent="0.3">
+      <c r="B39" s="20"/>
+      <c r="C39" s="19"/>
+      <c r="D39" s="10" t="s">
         <v>518</v>
       </c>
-      <c r="E38" s="10" t="s">
-        <v>462</v>
-      </c>
-      <c r="F38" s="10" t="s">
+      <c r="E39" s="10" t="s">
+        <v>464</v>
+      </c>
+      <c r="F39" s="10" t="s">
+        <v>465</v>
+      </c>
+      <c r="G39" s="11" t="s">
         <v>463</v>
       </c>
-      <c r="G38" s="11" t="s">
-        <v>461</v>
-      </c>
-      <c r="H38" s="11" t="s">
-        <v>539</v>
-      </c>
-    </row>
-    <row r="39" spans="2:8" x14ac:dyDescent="0.3">
-      <c r="B39" s="32"/>
-      <c r="C39" s="31"/>
-      <c r="D39" s="10" t="s">
-        <v>519</v>
-      </c>
-      <c r="E39" s="10" t="s">
-        <v>465</v>
-      </c>
-      <c r="F39" s="10" t="s">
-        <v>466</v>
-      </c>
-      <c r="G39" s="11" t="s">
-        <v>464</v>
-      </c>
       <c r="H39" s="11" t="s">
-        <v>539</v>
+        <v>538</v>
       </c>
     </row>
     <row r="40" spans="2:8" x14ac:dyDescent="0.3">
-      <c r="B40" s="32"/>
+      <c r="B40" s="20"/>
       <c r="C40" s="10" t="s">
         <v>3</v>
       </c>
@@ -4231,22 +4230,22 @@
         <v>7</v>
       </c>
       <c r="E40" s="10" t="s">
-        <v>467</v>
+        <v>466</v>
       </c>
       <c r="F40" s="10" t="s">
-        <v>502</v>
+        <v>501</v>
       </c>
       <c r="G40" s="11" t="s">
-        <v>583</v>
+        <v>582</v>
       </c>
       <c r="H40" s="11" t="s">
-        <v>567</v>
+        <v>566</v>
       </c>
     </row>
     <row r="41" spans="2:8" x14ac:dyDescent="0.3">
-      <c r="B41" s="32"/>
-      <c r="C41" s="31" t="s">
-        <v>520</v>
+      <c r="B41" s="20"/>
+      <c r="C41" s="19" t="s">
+        <v>519</v>
       </c>
       <c r="D41" s="10" t="s">
         <v>20</v>
@@ -4255,336 +4254,329 @@
         <v>11</v>
       </c>
       <c r="F41" s="10" t="s">
+        <v>467</v>
+      </c>
+      <c r="G41" s="11" t="s">
+        <v>583</v>
+      </c>
+      <c r="H41" s="11" t="s">
+        <v>538</v>
+      </c>
+    </row>
+    <row r="42" spans="2:8" x14ac:dyDescent="0.3">
+      <c r="B42" s="20"/>
+      <c r="C42" s="19"/>
+      <c r="D42" s="10" t="s">
+        <v>502</v>
+      </c>
+      <c r="E42" s="10" t="s">
         <v>468</v>
       </c>
-      <c r="G41" s="11" t="s">
+      <c r="F42" s="10" t="s">
+        <v>469</v>
+      </c>
+      <c r="G42" s="11" t="s">
         <v>584</v>
       </c>
-      <c r="H41" s="11" t="s">
-        <v>539</v>
-      </c>
-    </row>
-    <row r="42" spans="2:8" x14ac:dyDescent="0.3">
-      <c r="B42" s="32"/>
-      <c r="C42" s="31"/>
-      <c r="D42" s="10" t="s">
-        <v>503</v>
-      </c>
-      <c r="E42" s="10" t="s">
-        <v>469</v>
-      </c>
-      <c r="F42" s="10" t="s">
+      <c r="H42" s="11" t="s">
+        <v>538</v>
+      </c>
+    </row>
+    <row r="43" spans="2:8" x14ac:dyDescent="0.3">
+      <c r="B43" s="20"/>
+      <c r="C43" s="19" t="s">
+        <v>3</v>
+      </c>
+      <c r="D43" s="10" t="s">
+        <v>502</v>
+      </c>
+      <c r="E43" s="10" t="s">
         <v>470</v>
       </c>
-      <c r="G42" s="11" t="s">
+      <c r="F43" s="10" t="s">
+        <v>437</v>
+      </c>
+      <c r="G43" s="11" t="s">
         <v>585</v>
       </c>
-      <c r="H42" s="11" t="s">
-        <v>539</v>
-      </c>
-    </row>
-    <row r="43" spans="2:8" x14ac:dyDescent="0.3">
-      <c r="B43" s="32"/>
-      <c r="C43" s="31" t="s">
-        <v>3</v>
-      </c>
-      <c r="D43" s="10" t="s">
-        <v>503</v>
-      </c>
-      <c r="E43" s="10" t="s">
+      <c r="H43" s="11" t="s">
+        <v>567</v>
+      </c>
+    </row>
+    <row r="44" spans="2:8" x14ac:dyDescent="0.3">
+      <c r="B44" s="20"/>
+      <c r="C44" s="19"/>
+      <c r="D44" s="10" t="s">
         <v>471</v>
       </c>
-      <c r="F43" s="10" t="s">
-        <v>438</v>
-      </c>
-      <c r="G43" s="11" t="s">
+      <c r="E44" s="10" t="s">
+        <v>472</v>
+      </c>
+      <c r="F44" s="10" t="s">
+        <v>520</v>
+      </c>
+      <c r="G44" s="11" t="s">
         <v>586</v>
       </c>
-      <c r="H43" s="11" t="s">
-        <v>568</v>
-      </c>
-    </row>
-    <row r="44" spans="2:8" x14ac:dyDescent="0.3">
-      <c r="B44" s="32"/>
-      <c r="C44" s="31"/>
-      <c r="D44" s="10" t="s">
-        <v>472</v>
-      </c>
-      <c r="E44" s="10" t="s">
-        <v>473</v>
-      </c>
-      <c r="F44" s="10" t="s">
+      <c r="H44" s="11" t="s">
+        <v>587</v>
+      </c>
+    </row>
+    <row r="45" spans="2:8" x14ac:dyDescent="0.3">
+      <c r="B45" s="20"/>
+      <c r="C45" s="19" t="s">
         <v>521</v>
       </c>
-      <c r="G44" s="11" t="s">
-        <v>587</v>
-      </c>
-      <c r="H44" s="11" t="s">
+      <c r="D45" s="10" t="s">
+        <v>522</v>
+      </c>
+      <c r="E45" s="10" t="s">
+        <v>474</v>
+      </c>
+      <c r="F45" s="10" t="s">
+        <v>475</v>
+      </c>
+      <c r="G45" s="11" t="s">
         <v>588</v>
       </c>
-    </row>
-    <row r="45" spans="2:8" x14ac:dyDescent="0.3">
-      <c r="B45" s="32"/>
-      <c r="C45" s="31" t="s">
-        <v>522</v>
-      </c>
-      <c r="D45" s="10" t="s">
+      <c r="H45" s="11" t="s">
+        <v>589</v>
+      </c>
+    </row>
+    <row r="46" spans="2:8" x14ac:dyDescent="0.3">
+      <c r="B46" s="20"/>
+      <c r="C46" s="19"/>
+      <c r="D46" s="10" t="s">
         <v>523</v>
       </c>
-      <c r="E45" s="10" t="s">
-        <v>475</v>
-      </c>
-      <c r="F45" s="10" t="s">
+      <c r="E46" s="10" t="s">
         <v>476</v>
       </c>
-      <c r="G45" s="11" t="s">
-        <v>589</v>
-      </c>
-      <c r="H45" s="11" t="s">
+      <c r="F46" s="10" t="s">
+        <v>524</v>
+      </c>
+      <c r="G46" s="11" t="s">
         <v>590</v>
       </c>
-    </row>
-    <row r="46" spans="2:8" x14ac:dyDescent="0.3">
-      <c r="B46" s="32"/>
-      <c r="C46" s="31"/>
-      <c r="D46" s="10" t="s">
-        <v>524</v>
-      </c>
-      <c r="E46" s="10" t="s">
+      <c r="H46" s="11" t="s">
+        <v>591</v>
+      </c>
+    </row>
+    <row r="47" spans="2:8" x14ac:dyDescent="0.3">
+      <c r="B47" s="20"/>
+      <c r="C47" s="19" t="s">
+        <v>525</v>
+      </c>
+      <c r="D47" s="10" t="s">
         <v>477</v>
       </c>
-      <c r="F46" s="10" t="s">
-        <v>525</v>
-      </c>
-      <c r="G46" s="11" t="s">
-        <v>591</v>
-      </c>
-      <c r="H46" s="11" t="s">
+      <c r="E47" s="10" t="s">
+        <v>478</v>
+      </c>
+      <c r="F47" s="10" t="s">
+        <v>526</v>
+      </c>
+      <c r="G47" s="11" t="s">
         <v>592</v>
       </c>
-    </row>
-    <row r="47" spans="2:8" x14ac:dyDescent="0.3">
-      <c r="B47" s="32"/>
-      <c r="C47" s="31" t="s">
-        <v>526</v>
-      </c>
-      <c r="D47" s="10" t="s">
-        <v>478</v>
-      </c>
-      <c r="E47" s="10" t="s">
+      <c r="H47" s="11" t="s">
+        <v>593</v>
+      </c>
+    </row>
+    <row r="48" spans="2:8" x14ac:dyDescent="0.3">
+      <c r="B48" s="20"/>
+      <c r="C48" s="19"/>
+      <c r="D48" s="10" t="s">
+        <v>527</v>
+      </c>
+      <c r="E48" s="10" t="s">
         <v>479</v>
       </c>
-      <c r="F47" s="10" t="s">
-        <v>527</v>
-      </c>
-      <c r="G47" s="11" t="s">
-        <v>593</v>
-      </c>
-      <c r="H47" s="11" t="s">
-        <v>594</v>
-      </c>
-    </row>
-    <row r="48" spans="2:8" x14ac:dyDescent="0.3">
-      <c r="B48" s="32"/>
-      <c r="C48" s="31"/>
-      <c r="D48" s="10" t="s">
+      <c r="F48" s="10" t="s">
         <v>528</v>
-      </c>
-      <c r="E48" s="10" t="s">
-        <v>480</v>
-      </c>
-      <c r="F48" s="10" t="s">
-        <v>529</v>
       </c>
       <c r="G48" s="11" t="s">
         <v>101</v>
       </c>
       <c r="H48" s="11" t="s">
-        <v>595</v>
+        <v>594</v>
       </c>
     </row>
     <row r="49" spans="2:8" x14ac:dyDescent="0.3">
-      <c r="B49" s="32"/>
-      <c r="C49" s="31" t="s">
-        <v>677</v>
+      <c r="B49" s="20"/>
+      <c r="C49" s="19" t="s">
+        <v>676</v>
       </c>
       <c r="D49" s="10" t="s">
+        <v>641</v>
+      </c>
+      <c r="E49" s="10" t="s">
+        <v>650</v>
+      </c>
+      <c r="F49" s="10" t="s">
+        <v>651</v>
+      </c>
+      <c r="G49" s="11" t="s">
+        <v>652</v>
+      </c>
+      <c r="H49" s="11" t="s">
+        <v>653</v>
+      </c>
+    </row>
+    <row r="50" spans="2:8" x14ac:dyDescent="0.3">
+      <c r="B50" s="20"/>
+      <c r="C50" s="19"/>
+      <c r="D50" s="10" t="s">
         <v>642</v>
       </c>
-      <c r="E49" s="10" t="s">
-        <v>651</v>
-      </c>
-      <c r="F49" s="10" t="s">
+      <c r="E50" s="10" t="s">
+        <v>654</v>
+      </c>
+      <c r="F50" s="10" t="s">
+        <v>655</v>
+      </c>
+      <c r="G50" s="11" t="s">
         <v>652</v>
       </c>
-      <c r="G49" s="11" t="s">
-        <v>653</v>
-      </c>
-      <c r="H49" s="11" t="s">
-        <v>654</v>
-      </c>
-    </row>
-    <row r="50" spans="2:8" x14ac:dyDescent="0.3">
-      <c r="B50" s="32"/>
-      <c r="C50" s="31"/>
-      <c r="D50" s="10" t="s">
+      <c r="H50" s="11" t="s">
+        <v>656</v>
+      </c>
+    </row>
+    <row r="51" spans="2:8" x14ac:dyDescent="0.3">
+      <c r="B51" s="20"/>
+      <c r="C51" s="19"/>
+      <c r="D51" s="10" t="s">
         <v>643</v>
       </c>
-      <c r="E50" s="10" t="s">
-        <v>655</v>
-      </c>
-      <c r="F50" s="10" t="s">
-        <v>656</v>
-      </c>
-      <c r="G50" s="11" t="s">
-        <v>653</v>
-      </c>
-      <c r="H50" s="11" t="s">
+      <c r="E51" s="10" t="s">
         <v>657</v>
       </c>
-    </row>
-    <row r="51" spans="2:8" x14ac:dyDescent="0.3">
-      <c r="B51" s="32"/>
-      <c r="C51" s="31"/>
-      <c r="D51" s="10" t="s">
+      <c r="F51" s="10" t="s">
+        <v>658</v>
+      </c>
+      <c r="G51" s="11" t="s">
+        <v>659</v>
+      </c>
+      <c r="H51" s="11" t="s">
+        <v>573</v>
+      </c>
+    </row>
+    <row r="52" spans="2:8" ht="31.2" x14ac:dyDescent="0.3">
+      <c r="B52" s="20"/>
+      <c r="C52" s="19"/>
+      <c r="D52" s="10" t="s">
         <v>644</v>
       </c>
-      <c r="E51" s="10" t="s">
-        <v>658</v>
-      </c>
-      <c r="F51" s="10" t="s">
+      <c r="E52" s="10" t="s">
+        <v>660</v>
+      </c>
+      <c r="F52" s="10" t="s">
+        <v>661</v>
+      </c>
+      <c r="G52" s="11" t="s">
+        <v>652</v>
+      </c>
+      <c r="H52" s="11" t="s">
+        <v>662</v>
+      </c>
+    </row>
+    <row r="53" spans="2:8" x14ac:dyDescent="0.3">
+      <c r="B53" s="20"/>
+      <c r="C53" s="19"/>
+      <c r="D53" s="10" t="s">
+        <v>645</v>
+      </c>
+      <c r="E53" s="10" t="s">
+        <v>663</v>
+      </c>
+      <c r="F53" s="10" t="s">
+        <v>664</v>
+      </c>
+      <c r="G53" s="11" t="s">
         <v>659</v>
       </c>
-      <c r="G51" s="11" t="s">
-        <v>660</v>
-      </c>
-      <c r="H51" s="11" t="s">
-        <v>574</v>
-      </c>
-    </row>
-    <row r="52" spans="2:8" ht="31.2" x14ac:dyDescent="0.3">
-      <c r="B52" s="32"/>
-      <c r="C52" s="31"/>
-      <c r="D52" s="10" t="s">
-        <v>645</v>
-      </c>
-      <c r="E52" s="10" t="s">
-        <v>661</v>
-      </c>
-      <c r="F52" s="10" t="s">
-        <v>662</v>
-      </c>
-      <c r="G52" s="11" t="s">
-        <v>653</v>
-      </c>
-      <c r="H52" s="11" t="s">
-        <v>663</v>
-      </c>
-    </row>
-    <row r="53" spans="2:8" x14ac:dyDescent="0.3">
-      <c r="B53" s="32"/>
-      <c r="C53" s="31"/>
-      <c r="D53" s="10" t="s">
+      <c r="H53" s="11" t="s">
+        <v>572</v>
+      </c>
+    </row>
+    <row r="54" spans="2:8" x14ac:dyDescent="0.3">
+      <c r="B54" s="20"/>
+      <c r="C54" s="19"/>
+      <c r="D54" s="10" t="s">
         <v>646</v>
       </c>
-      <c r="E53" s="10" t="s">
-        <v>664</v>
-      </c>
-      <c r="F53" s="10" t="s">
+      <c r="E54" s="10" t="s">
         <v>665</v>
       </c>
-      <c r="G53" s="11" t="s">
-        <v>660</v>
-      </c>
-      <c r="H53" s="11" t="s">
-        <v>573</v>
-      </c>
-    </row>
-    <row r="54" spans="2:8" x14ac:dyDescent="0.3">
-      <c r="B54" s="32"/>
-      <c r="C54" s="31"/>
-      <c r="D54" s="10" t="s">
+      <c r="F54" s="10" t="s">
+        <v>666</v>
+      </c>
+      <c r="G54" s="11" t="s">
+        <v>659</v>
+      </c>
+      <c r="H54" s="11" t="s">
+        <v>667</v>
+      </c>
+    </row>
+    <row r="55" spans="2:8" x14ac:dyDescent="0.3">
+      <c r="B55" s="20"/>
+      <c r="C55" s="19"/>
+      <c r="D55" s="10" t="s">
         <v>647</v>
       </c>
-      <c r="E54" s="10" t="s">
-        <v>666</v>
-      </c>
-      <c r="F54" s="10" t="s">
-        <v>667</v>
-      </c>
-      <c r="G54" s="11" t="s">
-        <v>660</v>
-      </c>
-      <c r="H54" s="11" t="s">
+      <c r="E55" s="10" t="s">
         <v>668</v>
       </c>
-    </row>
-    <row r="55" spans="2:8" x14ac:dyDescent="0.3">
-      <c r="B55" s="32"/>
-      <c r="C55" s="31"/>
-      <c r="D55" s="10" t="s">
+      <c r="F55" s="10" t="s">
+        <v>669</v>
+      </c>
+      <c r="G55" s="11" t="s">
+        <v>659</v>
+      </c>
+      <c r="H55" s="11" t="s">
+        <v>670</v>
+      </c>
+    </row>
+    <row r="56" spans="2:8" x14ac:dyDescent="0.3">
+      <c r="B56" s="20"/>
+      <c r="C56" s="19"/>
+      <c r="D56" s="10" t="s">
         <v>648</v>
       </c>
-      <c r="E55" s="10" t="s">
-        <v>669</v>
-      </c>
-      <c r="F55" s="10" t="s">
-        <v>670</v>
-      </c>
-      <c r="G55" s="11" t="s">
-        <v>660</v>
-      </c>
-      <c r="H55" s="11" t="s">
+      <c r="E56" s="10" t="s">
         <v>671</v>
       </c>
-    </row>
-    <row r="56" spans="2:8" x14ac:dyDescent="0.3">
-      <c r="B56" s="32"/>
-      <c r="C56" s="31"/>
-      <c r="D56" s="10" t="s">
+      <c r="F56" s="10" t="s">
+        <v>672</v>
+      </c>
+      <c r="G56" s="11" t="s">
+        <v>659</v>
+      </c>
+      <c r="H56" s="11" t="s">
+        <v>673</v>
+      </c>
+    </row>
+    <row r="57" spans="2:8" x14ac:dyDescent="0.3">
+      <c r="B57" s="20"/>
+      <c r="C57" s="19"/>
+      <c r="D57" s="10" t="s">
         <v>649</v>
       </c>
-      <c r="E56" s="10" t="s">
-        <v>672</v>
-      </c>
-      <c r="F56" s="10" t="s">
+      <c r="E57" s="10" t="s">
+        <v>674</v>
+      </c>
+      <c r="F57" s="10" t="s">
+        <v>675</v>
+      </c>
+      <c r="G57" s="11" t="s">
+        <v>659</v>
+      </c>
+      <c r="H57" s="11" t="s">
         <v>673</v>
-      </c>
-      <c r="G56" s="11" t="s">
-        <v>660</v>
-      </c>
-      <c r="H56" s="11" t="s">
-        <v>674</v>
-      </c>
-    </row>
-    <row r="57" spans="2:8" x14ac:dyDescent="0.3">
-      <c r="B57" s="32"/>
-      <c r="C57" s="31"/>
-      <c r="D57" s="10" t="s">
-        <v>650</v>
-      </c>
-      <c r="E57" s="10" t="s">
-        <v>675</v>
-      </c>
-      <c r="F57" s="10" t="s">
-        <v>676</v>
-      </c>
-      <c r="G57" s="11" t="s">
-        <v>660</v>
-      </c>
-      <c r="H57" s="11" t="s">
-        <v>674</v>
       </c>
     </row>
   </sheetData>
   <mergeCells count="17">
-    <mergeCell ref="C49:C57"/>
-    <mergeCell ref="B38:B57"/>
-    <mergeCell ref="C38:C39"/>
-    <mergeCell ref="C41:C42"/>
-    <mergeCell ref="C43:C44"/>
-    <mergeCell ref="C45:C46"/>
-    <mergeCell ref="C47:C48"/>
     <mergeCell ref="C22:C24"/>
     <mergeCell ref="C25:C28"/>
     <mergeCell ref="C32:C35"/>
@@ -4595,6 +4587,13 @@
     <mergeCell ref="C13:C15"/>
     <mergeCell ref="C16:C17"/>
     <mergeCell ref="C18:C19"/>
+    <mergeCell ref="C49:C57"/>
+    <mergeCell ref="B38:B57"/>
+    <mergeCell ref="C38:C39"/>
+    <mergeCell ref="C41:C42"/>
+    <mergeCell ref="C43:C44"/>
+    <mergeCell ref="C45:C46"/>
+    <mergeCell ref="C47:C48"/>
   </mergeCells>
   <conditionalFormatting sqref="B3:H21">
     <cfRule type="colorScale" priority="1">
@@ -4626,12 +4625,12 @@
     <col min="7" max="16384" width="8.88671875" style="3"/>
   </cols>
   <sheetData>
-    <row r="2" spans="2:6" s="3" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="2" spans="2:6" x14ac:dyDescent="0.3">
       <c r="B2" s="1" t="s">
-        <v>413</v>
+        <v>412</v>
       </c>
       <c r="C2" s="1" t="s">
-        <v>481</v>
+        <v>480</v>
       </c>
       <c r="D2" s="1" t="s">
         <v>0</v>
@@ -4643,259 +4642,259 @@
         <v>234</v>
       </c>
     </row>
-    <row r="3" spans="2:6" s="3" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="3" spans="2:6" x14ac:dyDescent="0.3">
       <c r="B3" s="2" t="s">
+        <v>677</v>
+      </c>
+      <c r="C3" s="2" t="s">
         <v>678</v>
-      </c>
-      <c r="C3" s="2" t="s">
-        <v>679</v>
       </c>
       <c r="D3" s="2" t="s">
         <v>65</v>
       </c>
       <c r="E3" s="2" t="s">
+        <v>679</v>
+      </c>
+      <c r="F3" s="2" t="s">
         <v>680</v>
       </c>
-      <c r="F3" s="2" t="s">
-        <v>681</v>
-      </c>
-    </row>
-    <row r="4" spans="2:6" s="3" customFormat="1" x14ac:dyDescent="0.3">
+    </row>
+    <row r="4" spans="2:6" x14ac:dyDescent="0.3">
       <c r="B4" s="2" t="s">
+        <v>677</v>
+      </c>
+      <c r="C4" s="2" t="s">
         <v>678</v>
-      </c>
-      <c r="C4" s="2" t="s">
-        <v>679</v>
       </c>
       <c r="D4" s="2" t="s">
         <v>67</v>
       </c>
       <c r="E4" s="2" t="s">
+        <v>681</v>
+      </c>
+      <c r="F4" s="2" t="s">
         <v>682</v>
       </c>
-      <c r="F4" s="2" t="s">
-        <v>683</v>
-      </c>
-    </row>
-    <row r="5" spans="2:6" s="3" customFormat="1" x14ac:dyDescent="0.3">
+    </row>
+    <row r="5" spans="2:6" x14ac:dyDescent="0.3">
       <c r="B5" s="2" t="s">
         <v>12</v>
       </c>
       <c r="C5" s="2" t="s">
-        <v>684</v>
+        <v>683</v>
       </c>
       <c r="D5" s="2" t="s">
         <v>63</v>
       </c>
       <c r="E5" s="2" t="s">
+        <v>684</v>
+      </c>
+      <c r="F5" s="2" t="s">
         <v>685</v>
       </c>
-      <c r="F5" s="2" t="s">
+    </row>
+    <row r="6" spans="2:6" x14ac:dyDescent="0.3">
+      <c r="B6" s="2" t="s">
+        <v>677</v>
+      </c>
+      <c r="C6" s="2" t="s">
         <v>686</v>
       </c>
-    </row>
-    <row r="6" spans="2:6" s="3" customFormat="1" x14ac:dyDescent="0.3">
-      <c r="B6" s="2" t="s">
-        <v>678</v>
-      </c>
-      <c r="C6" s="2" t="s">
+      <c r="D6" s="2" t="s">
         <v>687</v>
       </c>
-      <c r="D6" s="2" t="s">
+      <c r="E6" s="2" t="s">
         <v>688</v>
       </c>
-      <c r="E6" s="2" t="s">
+      <c r="F6" s="2" t="s">
         <v>689</v>
       </c>
-      <c r="F6" s="2" t="s">
+    </row>
+    <row r="7" spans="2:6" x14ac:dyDescent="0.3">
+      <c r="B7" s="2" t="s">
+        <v>677</v>
+      </c>
+      <c r="C7" s="2" t="s">
+        <v>686</v>
+      </c>
+      <c r="D7" s="2" t="s">
         <v>690</v>
       </c>
-    </row>
-    <row r="7" spans="2:6" s="3" customFormat="1" x14ac:dyDescent="0.3">
-      <c r="B7" s="2" t="s">
-        <v>678</v>
-      </c>
-      <c r="C7" s="2" t="s">
+      <c r="E7" s="2" t="s">
+        <v>691</v>
+      </c>
+      <c r="F7" s="2" t="s">
+        <v>692</v>
+      </c>
+    </row>
+    <row r="8" spans="2:6" x14ac:dyDescent="0.3">
+      <c r="B8" s="2" t="s">
+        <v>677</v>
+      </c>
+      <c r="C8" s="2" t="s">
+        <v>693</v>
+      </c>
+      <c r="D8" s="2" t="s">
         <v>687</v>
       </c>
-      <c r="D7" s="2" t="s">
-        <v>691</v>
-      </c>
-      <c r="E7" s="2" t="s">
-        <v>692</v>
-      </c>
-      <c r="F7" s="2" t="s">
-        <v>693</v>
-      </c>
-    </row>
-    <row r="8" spans="2:6" s="3" customFormat="1" x14ac:dyDescent="0.3">
-      <c r="B8" s="2" t="s">
-        <v>678</v>
-      </c>
-      <c r="C8" s="2" t="s">
+      <c r="E8" s="2" t="s">
         <v>694</v>
       </c>
-      <c r="D8" s="2" t="s">
-        <v>688</v>
-      </c>
-      <c r="E8" s="2" t="s">
+      <c r="F8" s="2" t="s">
         <v>695</v>
       </c>
-      <c r="F8" s="2" t="s">
+    </row>
+    <row r="9" spans="2:6" x14ac:dyDescent="0.3">
+      <c r="B9" s="2" t="s">
         <v>696</v>
       </c>
-    </row>
-    <row r="9" spans="2:6" s="3" customFormat="1" x14ac:dyDescent="0.3">
-      <c r="B9" s="2" t="s">
+      <c r="C9" s="2" t="s">
         <v>697</v>
       </c>
-      <c r="C9" s="2" t="s">
+      <c r="D9" s="2" t="s">
         <v>698</v>
       </c>
-      <c r="D9" s="2" t="s">
+      <c r="E9" s="2" t="s">
         <v>699</v>
       </c>
-      <c r="E9" s="2" t="s">
+      <c r="F9" s="2" t="s">
         <v>700</v>
       </c>
-      <c r="F9" s="2" t="s">
+    </row>
+    <row r="10" spans="2:6" x14ac:dyDescent="0.3">
+      <c r="B10" s="2" t="s">
         <v>701</v>
       </c>
-    </row>
-    <row r="10" spans="2:6" s="3" customFormat="1" x14ac:dyDescent="0.3">
-      <c r="B10" s="2" t="s">
+      <c r="C10" s="2" t="s">
         <v>702</v>
-      </c>
-      <c r="C10" s="2" t="s">
-        <v>703</v>
       </c>
       <c r="D10" s="2" t="s">
         <v>89</v>
       </c>
       <c r="E10" s="2" t="s">
+        <v>703</v>
+      </c>
+      <c r="F10" s="2" t="s">
         <v>704</v>
       </c>
-      <c r="F10" s="2" t="s">
+    </row>
+    <row r="11" spans="2:6" x14ac:dyDescent="0.3">
+      <c r="B11" s="2" t="s">
+        <v>701</v>
+      </c>
+      <c r="C11" s="2" t="s">
         <v>705</v>
       </c>
-    </row>
-    <row r="11" spans="2:6" s="3" customFormat="1" x14ac:dyDescent="0.3">
-      <c r="B11" s="2" t="s">
-        <v>702</v>
-      </c>
-      <c r="C11" s="2" t="s">
+      <c r="D11" s="2" t="s">
         <v>706</v>
       </c>
-      <c r="D11" s="2" t="s">
+      <c r="E11" s="2" t="s">
         <v>707</v>
       </c>
-      <c r="E11" s="2" t="s">
+      <c r="F11" s="2" t="s">
         <v>708</v>
       </c>
-      <c r="F11" s="2" t="s">
+    </row>
+    <row r="12" spans="2:6" x14ac:dyDescent="0.3">
+      <c r="B12" s="2" t="s">
+        <v>701</v>
+      </c>
+      <c r="C12" s="2" t="s">
         <v>709</v>
-      </c>
-    </row>
-    <row r="12" spans="2:6" s="3" customFormat="1" x14ac:dyDescent="0.3">
-      <c r="B12" s="2" t="s">
-        <v>702</v>
-      </c>
-      <c r="C12" s="2" t="s">
-        <v>710</v>
       </c>
       <c r="D12" s="2" t="s">
         <v>63</v>
       </c>
       <c r="E12" s="2" t="s">
+        <v>710</v>
+      </c>
+      <c r="F12" s="2" t="s">
         <v>711</v>
       </c>
-      <c r="F12" s="2" t="s">
+    </row>
+    <row r="13" spans="2:6" x14ac:dyDescent="0.3">
+      <c r="B13" s="2" t="s">
         <v>712</v>
       </c>
-    </row>
-    <row r="13" spans="2:6" s="3" customFormat="1" x14ac:dyDescent="0.3">
-      <c r="B13" s="2" t="s">
+      <c r="C13" s="2" t="s">
         <v>713</v>
-      </c>
-      <c r="C13" s="2" t="s">
-        <v>714</v>
       </c>
       <c r="D13" s="2" t="s">
         <v>69</v>
       </c>
       <c r="E13" s="2" t="s">
+        <v>714</v>
+      </c>
+      <c r="F13" s="2" t="s">
         <v>715</v>
       </c>
-      <c r="F13" s="2" t="s">
+    </row>
+    <row r="14" spans="2:6" x14ac:dyDescent="0.3">
+      <c r="B14" s="2" t="s">
+        <v>712</v>
+      </c>
+      <c r="C14" s="2" t="s">
         <v>716</v>
       </c>
-    </row>
-    <row r="14" spans="2:6" s="3" customFormat="1" x14ac:dyDescent="0.3">
-      <c r="B14" s="2" t="s">
-        <v>713</v>
-      </c>
-      <c r="C14" s="2" t="s">
+      <c r="D14" s="2" t="s">
         <v>717</v>
       </c>
-      <c r="D14" s="2" t="s">
+      <c r="E14" s="2" t="s">
         <v>718</v>
       </c>
-      <c r="E14" s="2" t="s">
+      <c r="F14" s="2" t="s">
         <v>719</v>
       </c>
-      <c r="F14" s="2" t="s">
+    </row>
+    <row r="15" spans="2:6" x14ac:dyDescent="0.3">
+      <c r="B15" s="2" t="s">
+        <v>677</v>
+      </c>
+      <c r="C15" s="2" t="s">
         <v>720</v>
       </c>
-    </row>
-    <row r="15" spans="2:6" s="3" customFormat="1" x14ac:dyDescent="0.3">
-      <c r="B15" s="2" t="s">
-        <v>678</v>
-      </c>
-      <c r="C15" s="2" t="s">
+      <c r="D15" s="2" t="s">
         <v>721</v>
       </c>
-      <c r="D15" s="2" t="s">
+      <c r="E15" s="2" t="s">
         <v>722</v>
       </c>
-      <c r="E15" s="2" t="s">
+      <c r="F15" s="2" t="s">
         <v>723</v>
       </c>
-      <c r="F15" s="2" t="s">
+    </row>
+    <row r="16" spans="2:6" x14ac:dyDescent="0.3">
+      <c r="B16" s="2" t="s">
         <v>724</v>
       </c>
-    </row>
-    <row r="16" spans="2:6" s="3" customFormat="1" x14ac:dyDescent="0.3">
-      <c r="B16" s="2" t="s">
+      <c r="C16" s="2" t="s">
         <v>725</v>
       </c>
-      <c r="C16" s="2" t="s">
+      <c r="D16" s="2" t="s">
         <v>726</v>
       </c>
-      <c r="D16" s="2" t="s">
+      <c r="E16" s="2" t="s">
         <v>727</v>
       </c>
-      <c r="E16" s="2" t="s">
+      <c r="F16" s="2" t="s">
         <v>728</v>
       </c>
-      <c r="F16" s="2" t="s">
+    </row>
+    <row r="17" spans="2:6" x14ac:dyDescent="0.3">
+      <c r="B17" s="2" t="s">
+        <v>724</v>
+      </c>
+      <c r="C17" s="2" t="s">
         <v>729</v>
-      </c>
-    </row>
-    <row r="17" spans="2:6" s="3" customFormat="1" x14ac:dyDescent="0.3">
-      <c r="B17" s="2" t="s">
-        <v>725</v>
-      </c>
-      <c r="C17" s="2" t="s">
-        <v>730</v>
       </c>
       <c r="D17" s="2" t="s">
         <v>91</v>
       </c>
       <c r="E17" s="2" t="s">
+        <v>730</v>
+      </c>
+      <c r="F17" s="2" t="s">
         <v>731</v>
-      </c>
-      <c r="F17" s="2" t="s">
-        <v>732</v>
       </c>
     </row>
   </sheetData>
@@ -5046,7 +5045,7 @@
         <v>148</v>
       </c>
       <c r="E3" s="2" t="s">
-        <v>377</v>
+        <v>376</v>
       </c>
     </row>
     <row r="4" spans="2:5" x14ac:dyDescent="0.3">
@@ -5058,7 +5057,7 @@
         <v>150</v>
       </c>
       <c r="E4" s="2" t="s">
-        <v>378</v>
+        <v>377</v>
       </c>
     </row>
     <row r="5" spans="2:5" x14ac:dyDescent="0.3">
@@ -5070,7 +5069,7 @@
         <v>152</v>
       </c>
       <c r="E5" s="2" t="s">
-        <v>379</v>
+        <v>378</v>
       </c>
     </row>
     <row r="6" spans="2:5" x14ac:dyDescent="0.3">
@@ -5084,7 +5083,7 @@
         <v>155</v>
       </c>
       <c r="E6" s="2" t="s">
-        <v>380</v>
+        <v>379</v>
       </c>
     </row>
     <row r="7" spans="2:5" x14ac:dyDescent="0.3">
@@ -5096,7 +5095,7 @@
         <v>157</v>
       </c>
       <c r="E7" s="2" t="s">
-        <v>381</v>
+        <v>380</v>
       </c>
     </row>
     <row r="8" spans="2:5" x14ac:dyDescent="0.3">
@@ -5108,7 +5107,7 @@
         <v>159</v>
       </c>
       <c r="E8" s="2" t="s">
-        <v>382</v>
+        <v>381</v>
       </c>
     </row>
     <row r="9" spans="2:5" x14ac:dyDescent="0.3">
@@ -5120,7 +5119,7 @@
         <v>161</v>
       </c>
       <c r="E9" s="2" t="s">
-        <v>383</v>
+        <v>382</v>
       </c>
     </row>
     <row r="10" spans="2:5" x14ac:dyDescent="0.3">
@@ -5134,7 +5133,7 @@
         <v>164</v>
       </c>
       <c r="E10" s="2" t="s">
-        <v>384</v>
+        <v>383</v>
       </c>
     </row>
     <row r="11" spans="2:5" x14ac:dyDescent="0.3">
@@ -5146,7 +5145,7 @@
         <v>166</v>
       </c>
       <c r="E11" s="2" t="s">
-        <v>385</v>
+        <v>384</v>
       </c>
     </row>
     <row r="12" spans="2:5" x14ac:dyDescent="0.3">
@@ -5158,7 +5157,7 @@
         <v>168</v>
       </c>
       <c r="E12" s="2" t="s">
-        <v>386</v>
+        <v>385</v>
       </c>
     </row>
     <row r="13" spans="2:5" x14ac:dyDescent="0.3">
@@ -5170,7 +5169,7 @@
         <v>170</v>
       </c>
       <c r="E13" s="2" t="s">
-        <v>387</v>
+        <v>386</v>
       </c>
     </row>
     <row r="14" spans="2:5" x14ac:dyDescent="0.3">
@@ -5182,7 +5181,7 @@
         <v>172</v>
       </c>
       <c r="E14" s="2" t="s">
-        <v>388</v>
+        <v>387</v>
       </c>
     </row>
     <row r="15" spans="2:5" x14ac:dyDescent="0.3">
@@ -5196,7 +5195,7 @@
         <v>175</v>
       </c>
       <c r="E15" s="2" t="s">
-        <v>389</v>
+        <v>388</v>
       </c>
     </row>
     <row r="16" spans="2:5" x14ac:dyDescent="0.3">
@@ -5208,7 +5207,7 @@
         <v>177</v>
       </c>
       <c r="E16" s="2" t="s">
-        <v>390</v>
+        <v>389</v>
       </c>
     </row>
     <row r="17" spans="2:5" x14ac:dyDescent="0.3">
@@ -5220,7 +5219,7 @@
         <v>179</v>
       </c>
       <c r="E17" s="2" t="s">
-        <v>391</v>
+        <v>390</v>
       </c>
     </row>
     <row r="18" spans="2:5" x14ac:dyDescent="0.3">
@@ -5234,7 +5233,7 @@
         <v>182</v>
       </c>
       <c r="E18" s="2" t="s">
-        <v>392</v>
+        <v>391</v>
       </c>
     </row>
     <row r="19" spans="2:5" x14ac:dyDescent="0.3">
@@ -5246,7 +5245,7 @@
         <v>184</v>
       </c>
       <c r="E19" s="2" t="s">
-        <v>393</v>
+        <v>392</v>
       </c>
     </row>
     <row r="20" spans="2:5" x14ac:dyDescent="0.3">
@@ -5258,7 +5257,7 @@
         <v>186</v>
       </c>
       <c r="E20" s="2" t="s">
-        <v>394</v>
+        <v>393</v>
       </c>
     </row>
     <row r="21" spans="2:5" x14ac:dyDescent="0.3">
@@ -5272,7 +5271,7 @@
         <v>189</v>
       </c>
       <c r="E21" s="2" t="s">
-        <v>395</v>
+        <v>394</v>
       </c>
     </row>
     <row r="22" spans="2:5" x14ac:dyDescent="0.3">
@@ -5284,7 +5283,7 @@
         <v>191</v>
       </c>
       <c r="E22" s="2" t="s">
-        <v>396</v>
+        <v>395</v>
       </c>
     </row>
     <row r="23" spans="2:5" x14ac:dyDescent="0.3">
@@ -5298,7 +5297,7 @@
         <v>194</v>
       </c>
       <c r="E23" s="2" t="s">
-        <v>397</v>
+        <v>396</v>
       </c>
     </row>
     <row r="24" spans="2:5" x14ac:dyDescent="0.3">
@@ -5312,7 +5311,7 @@
         <v>197</v>
       </c>
       <c r="E24" s="2" t="s">
-        <v>398</v>
+        <v>397</v>
       </c>
     </row>
     <row r="25" spans="2:5" x14ac:dyDescent="0.3">
@@ -5326,7 +5325,7 @@
         <v>200</v>
       </c>
       <c r="E25" s="2" t="s">
-        <v>399</v>
+        <v>398</v>
       </c>
     </row>
     <row r="26" spans="2:5" x14ac:dyDescent="0.3">
@@ -5338,7 +5337,7 @@
         <v>202</v>
       </c>
       <c r="E26" s="2" t="s">
-        <v>400</v>
+        <v>399</v>
       </c>
     </row>
     <row r="27" spans="2:5" x14ac:dyDescent="0.3">
@@ -5352,7 +5351,7 @@
         <v>205</v>
       </c>
       <c r="E27" s="2" t="s">
-        <v>401</v>
+        <v>400</v>
       </c>
     </row>
     <row r="28" spans="2:5" x14ac:dyDescent="0.3">
@@ -5364,7 +5363,7 @@
         <v>207</v>
       </c>
       <c r="E28" s="2" t="s">
-        <v>402</v>
+        <v>401</v>
       </c>
     </row>
     <row r="29" spans="2:5" x14ac:dyDescent="0.3">
@@ -5376,7 +5375,7 @@
         <v>209</v>
       </c>
       <c r="E29" s="2" t="s">
-        <v>403</v>
+        <v>402</v>
       </c>
     </row>
     <row r="30" spans="2:5" x14ac:dyDescent="0.3">
@@ -5388,7 +5387,7 @@
         <v>211</v>
       </c>
       <c r="E30" s="2" t="s">
-        <v>404</v>
+        <v>403</v>
       </c>
     </row>
     <row r="31" spans="2:5" x14ac:dyDescent="0.3">
@@ -5400,7 +5399,7 @@
         <v>213</v>
       </c>
       <c r="E31" s="2" t="s">
-        <v>405</v>
+        <v>404</v>
       </c>
     </row>
     <row r="32" spans="2:5" x14ac:dyDescent="0.3">
@@ -5412,7 +5411,7 @@
         <v>215</v>
       </c>
       <c r="E32" s="2" t="s">
-        <v>406</v>
+        <v>405</v>
       </c>
     </row>
     <row r="33" spans="2:5" x14ac:dyDescent="0.3">
@@ -5424,7 +5423,7 @@
         <v>217</v>
       </c>
       <c r="E33" s="2" t="s">
-        <v>407</v>
+        <v>406</v>
       </c>
     </row>
     <row r="34" spans="2:5" x14ac:dyDescent="0.3">
@@ -5436,7 +5435,7 @@
         <v>219</v>
       </c>
       <c r="E34" s="2" t="s">
-        <v>408</v>
+        <v>407</v>
       </c>
     </row>
     <row r="35" spans="2:5" x14ac:dyDescent="0.3">
@@ -5448,7 +5447,7 @@
         <v>221</v>
       </c>
       <c r="E35" s="2" t="s">
-        <v>409</v>
+        <v>408</v>
       </c>
     </row>
     <row r="36" spans="2:5" x14ac:dyDescent="0.3">
@@ -5460,7 +5459,7 @@
         <v>223</v>
       </c>
       <c r="E36" s="2" t="s">
-        <v>410</v>
+        <v>409</v>
       </c>
     </row>
     <row r="37" spans="2:5" x14ac:dyDescent="0.3">
@@ -5474,7 +5473,7 @@
         <v>226</v>
       </c>
       <c r="E37" s="2" t="s">
-        <v>411</v>
+        <v>410</v>
       </c>
     </row>
     <row r="38" spans="2:5" x14ac:dyDescent="0.3">
@@ -5488,7 +5487,7 @@
         <v>229</v>
       </c>
       <c r="E38" s="2" t="s">
-        <v>412</v>
+        <v>411</v>
       </c>
     </row>
   </sheetData>
@@ -5518,10 +5517,10 @@
   <sheetData>
     <row r="2" spans="2:4" ht="15.6" x14ac:dyDescent="0.3">
       <c r="B2" s="1" t="s">
+        <v>610</v>
+      </c>
+      <c r="C2" s="1" t="s">
         <v>611</v>
-      </c>
-      <c r="C2" s="1" t="s">
-        <v>612</v>
       </c>
       <c r="D2" s="1" t="s">
         <v>29</v>
@@ -5532,10 +5531,10 @@
         <v>147</v>
       </c>
       <c r="C3" s="2" t="s">
+        <v>612</v>
+      </c>
+      <c r="D3" s="2" t="s">
         <v>613</v>
-      </c>
-      <c r="D3" s="2" t="s">
-        <v>614</v>
       </c>
     </row>
     <row r="4" spans="2:4" ht="15.6" x14ac:dyDescent="0.3">
@@ -5543,10 +5542,10 @@
         <v>149</v>
       </c>
       <c r="C4" s="2" t="s">
+        <v>614</v>
+      </c>
+      <c r="D4" s="2" t="s">
         <v>615</v>
-      </c>
-      <c r="D4" s="2" t="s">
-        <v>616</v>
       </c>
     </row>
     <row r="5" spans="2:4" ht="15.6" x14ac:dyDescent="0.3">
@@ -5554,10 +5553,10 @@
         <v>154</v>
       </c>
       <c r="C5" s="2" t="s">
+        <v>616</v>
+      </c>
+      <c r="D5" s="2" t="s">
         <v>617</v>
-      </c>
-      <c r="D5" s="2" t="s">
-        <v>618</v>
       </c>
     </row>
     <row r="6" spans="2:4" ht="15.6" x14ac:dyDescent="0.3">
@@ -5565,10 +5564,10 @@
         <v>156</v>
       </c>
       <c r="C6" s="2" t="s">
+        <v>618</v>
+      </c>
+      <c r="D6" s="2" t="s">
         <v>619</v>
-      </c>
-      <c r="D6" s="2" t="s">
-        <v>620</v>
       </c>
     </row>
     <row r="7" spans="2:4" ht="15.6" x14ac:dyDescent="0.3">
@@ -5576,10 +5575,10 @@
         <v>163</v>
       </c>
       <c r="C7" s="2" t="s">
+        <v>620</v>
+      </c>
+      <c r="D7" s="2" t="s">
         <v>621</v>
-      </c>
-      <c r="D7" s="2" t="s">
-        <v>622</v>
       </c>
     </row>
     <row r="8" spans="2:4" ht="15.6" x14ac:dyDescent="0.3">
@@ -5587,10 +5586,10 @@
         <v>165</v>
       </c>
       <c r="C8" s="2" t="s">
+        <v>622</v>
+      </c>
+      <c r="D8" s="2" t="s">
         <v>623</v>
-      </c>
-      <c r="D8" s="2" t="s">
-        <v>624</v>
       </c>
     </row>
     <row r="9" spans="2:4" ht="15.6" x14ac:dyDescent="0.3">
@@ -5598,10 +5597,10 @@
         <v>174</v>
       </c>
       <c r="C9" s="2" t="s">
+        <v>624</v>
+      </c>
+      <c r="D9" s="2" t="s">
         <v>625</v>
-      </c>
-      <c r="D9" s="2" t="s">
-        <v>626</v>
       </c>
     </row>
     <row r="10" spans="2:4" ht="15.6" x14ac:dyDescent="0.3">
@@ -5609,10 +5608,10 @@
         <v>176</v>
       </c>
       <c r="C10" s="2" t="s">
+        <v>626</v>
+      </c>
+      <c r="D10" s="2" t="s">
         <v>627</v>
-      </c>
-      <c r="D10" s="2" t="s">
-        <v>628</v>
       </c>
     </row>
     <row r="11" spans="2:4" ht="15.6" x14ac:dyDescent="0.3">
@@ -5620,10 +5619,10 @@
         <v>188</v>
       </c>
       <c r="C11" s="2" t="s">
+        <v>628</v>
+      </c>
+      <c r="D11" s="2" t="s">
         <v>629</v>
-      </c>
-      <c r="D11" s="2" t="s">
-        <v>630</v>
       </c>
     </row>
     <row r="12" spans="2:4" ht="15.6" x14ac:dyDescent="0.3">
@@ -5631,10 +5630,10 @@
         <v>181</v>
       </c>
       <c r="C12" s="2" t="s">
+        <v>630</v>
+      </c>
+      <c r="D12" s="2" t="s">
         <v>631</v>
-      </c>
-      <c r="D12" s="2" t="s">
-        <v>632</v>
       </c>
     </row>
     <row r="13" spans="2:4" ht="15.6" x14ac:dyDescent="0.3">
@@ -5642,10 +5641,10 @@
         <v>193</v>
       </c>
       <c r="C13" s="2" t="s">
+        <v>632</v>
+      </c>
+      <c r="D13" s="2" t="s">
         <v>633</v>
-      </c>
-      <c r="D13" s="2" t="s">
-        <v>634</v>
       </c>
     </row>
     <row r="14" spans="2:4" ht="15.6" x14ac:dyDescent="0.3">
@@ -5653,21 +5652,21 @@
         <v>196</v>
       </c>
       <c r="C14" s="2" t="s">
+        <v>634</v>
+      </c>
+      <c r="D14" s="2" t="s">
         <v>635</v>
-      </c>
-      <c r="D14" s="2" t="s">
-        <v>636</v>
       </c>
     </row>
     <row r="15" spans="2:4" ht="15.6" x14ac:dyDescent="0.3">
       <c r="B15" s="2" t="s">
+        <v>636</v>
+      </c>
+      <c r="C15" s="2" t="s">
         <v>637</v>
       </c>
-      <c r="C15" s="2" t="s">
+      <c r="D15" s="2" t="s">
         <v>638</v>
-      </c>
-      <c r="D15" s="2" t="s">
-        <v>639</v>
       </c>
     </row>
     <row r="16" spans="2:4" ht="15.6" x14ac:dyDescent="0.3">
@@ -5675,10 +5674,10 @@
         <v>183</v>
       </c>
       <c r="C16" s="2" t="s">
+        <v>639</v>
+      </c>
+      <c r="D16" s="2" t="s">
         <v>640</v>
-      </c>
-      <c r="D16" s="2" t="s">
-        <v>641</v>
       </c>
     </row>
   </sheetData>

</xml_diff>